<commit_message>
Expand formal paper output and solver status
</commit_message>
<xml_diff>
--- a/A_solution/outputs/A题_求解结果汇总.xlsx
+++ b/A_solution/outputs/A题_求解结果汇总.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1487,15 +1487,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>strict_milp_solver_available</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>problem4_solver_status</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>problem4_storage_e_nonnegative</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="C7" t="b">
+      <c r="C9" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add optional PuLP MILP storage solver
</commit_message>
<xml_diff>
--- a/A_solution/outputs/A题_求解结果汇总.xlsx
+++ b/A_solution/outputs/A题_求解结果汇总.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1487,7 +1487,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>strict_milp_solver_available</t>
+          <t>scipy_available</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>problem4_solver_status</t>
+          <t>pulp_available</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>False</t>
         </is>
       </c>
       <c r="C8" t="b">
@@ -1517,15 +1517,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>strict_milp_solver_available</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>problem4_solver_status</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>problem4_storage_e_nonnegative</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>20.0</t>
         </is>
       </c>
-      <c r="C9" t="b">
+      <c r="C11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -20269,7 +20299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:X25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20380,10 +20410,15 @@
       </c>
       <c r="V1" t="inlineStr">
         <is>
+          <t>solver_status</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
           <t>curtail_mwh</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>base_unserved_mwh</t>
         </is>
@@ -20461,10 +20496,15 @@
       <c r="U2" t="n">
         <v>5</v>
       </c>
-      <c r="V2" t="n">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
         <v>112.8358942581749</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20540,10 +20580,15 @@
       <c r="U3" t="n">
         <v>5</v>
       </c>
-      <c r="V3" t="n">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
         <v>2.450200000000002</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20619,10 +20664,15 @@
       <c r="U4" t="n">
         <v>5</v>
       </c>
-      <c r="V4" t="n">
-        <v>0</v>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20698,10 +20748,15 @@
       <c r="U5" t="n">
         <v>5</v>
       </c>
-      <c r="V5" t="n">
-        <v>0</v>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20777,10 +20832,15 @@
       <c r="U6" t="n">
         <v>5</v>
       </c>
-      <c r="V6" t="n">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
         <v>67.20108868896887</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20856,10 +20916,15 @@
       <c r="U7" t="n">
         <v>5</v>
       </c>
-      <c r="V7" t="n">
-        <v>0</v>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20935,10 +21000,15 @@
       <c r="U8" t="n">
         <v>5</v>
       </c>
-      <c r="V8" t="n">
-        <v>0</v>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21014,10 +21084,15 @@
       <c r="U9" t="n">
         <v>5</v>
       </c>
-      <c r="V9" t="n">
-        <v>0</v>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21093,10 +21168,15 @@
       <c r="U10" t="n">
         <v>5</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W10" t="n">
         <v>103.8897580185268</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21172,10 +21252,15 @@
       <c r="U11" t="n">
         <v>5</v>
       </c>
-      <c r="V11" t="n">
-        <v>0</v>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21251,10 +21336,15 @@
       <c r="U12" t="n">
         <v>5</v>
       </c>
-      <c r="V12" t="n">
-        <v>0</v>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21330,10 +21420,15 @@
       <c r="U13" t="n">
         <v>5</v>
       </c>
-      <c r="V13" t="n">
-        <v>0</v>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21409,10 +21504,15 @@
       <c r="U14" t="n">
         <v>5</v>
       </c>
-      <c r="V14" t="n">
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W14" t="n">
         <v>151.1617553556355</v>
       </c>
-      <c r="W14" t="n">
+      <c r="X14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21488,10 +21588,15 @@
       <c r="U15" t="n">
         <v>5</v>
       </c>
-      <c r="V15" t="n">
-        <v>0</v>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21567,10 +21672,15 @@
       <c r="U16" t="n">
         <v>5</v>
       </c>
-      <c r="V16" t="n">
-        <v>0</v>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21646,10 +21756,15 @@
       <c r="U17" t="n">
         <v>5</v>
       </c>
-      <c r="V17" t="n">
-        <v>0</v>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21725,10 +21840,15 @@
       <c r="U18" t="n">
         <v>5</v>
       </c>
-      <c r="V18" t="n">
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W18" t="n">
         <v>136.14439980008</v>
       </c>
-      <c r="W18" t="n">
+      <c r="X18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21804,10 +21924,15 @@
       <c r="U19" t="n">
         <v>5</v>
       </c>
-      <c r="V19" t="n">
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
         <v>0.7421999999999969</v>
       </c>
-      <c r="W19" t="n">
+      <c r="X19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21883,10 +22008,15 @@
       <c r="U20" t="n">
         <v>5</v>
       </c>
-      <c r="V20" t="n">
-        <v>0</v>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W20" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21962,10 +22092,15 @@
       <c r="U21" t="n">
         <v>5</v>
       </c>
-      <c r="V21" t="n">
-        <v>0</v>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W21" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22041,10 +22176,15 @@
       <c r="U22" t="n">
         <v>5</v>
       </c>
-      <c r="V22" t="n">
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
+      </c>
+      <c r="W22" t="n">
         <v>68.40251787449543</v>
       </c>
-      <c r="W22" t="n">
+      <c r="X22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22120,10 +22260,15 @@
       <c r="U23" t="n">
         <v>5</v>
       </c>
-      <c r="V23" t="n">
-        <v>0</v>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W23" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22199,10 +22344,15 @@
       <c r="U24" t="n">
         <v>5</v>
       </c>
-      <c r="V24" t="n">
-        <v>0</v>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W24" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22278,10 +22428,15 @@
       <c r="U25" t="n">
         <v>5</v>
       </c>
-      <c r="V25" t="n">
-        <v>0</v>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>discrete_storage_fallback</t>
+        </is>
       </c>
       <c r="W25" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize strict MILP outputs
</commit_message>
<xml_diff>
--- a/A_solution/outputs/A题_求解结果汇总.xlsx
+++ b/A_solution/outputs/A题_求解结果汇总.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem1_hourly" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem1_summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem2_scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem2_typical_summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem2_year_summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem3_scenarios" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem3_year_summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem4_no_storage" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem4_storage" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="problem4_storage_config" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="validation_checks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="problem1_hourly" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="problem1_summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="problem2_scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="problem2_typical_summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="problem2_year_summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="problem3_scenarios" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="problem3_year_summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="problem4_no_storage" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="problem4_storage" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="problem4_storage_config" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="validation_checks" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1369,13 +1369,13 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>42648772.66080074</v>
+        <v>42682238.13736948</v>
       </c>
       <c r="G2" t="n">
-        <v>10044.42654055611</v>
+        <v>10064.49378615</v>
       </c>
       <c r="H2" t="n">
-        <v>4246.013696112858</v>
+        <v>4240.872819267431</v>
       </c>
     </row>
   </sheetData>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C7" t="b">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C8" t="b">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C9" t="b">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp</t>
         </is>
       </c>
       <c r="C10" t="b">
@@ -20441,10 +20441,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>42.11672526889501</v>
+        <v>42.18619865</v>
       </c>
       <c r="E2" t="n">
-        <v>643.3346995530476</v>
+        <v>644.2957469916666</v>
       </c>
       <c r="F2" t="n">
         <v>761.7639999999999</v>
@@ -20456,19 +20456,19 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8445328206019813</v>
+        <v>0.8457944284472182</v>
       </c>
       <c r="J2" t="n">
-        <v>1.184086604576483</v>
+        <v>1.182320391771657</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2445328206019813</v>
+        <v>0.2457944284472182</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8840866045764828</v>
+        <v>0.8823203917716573</v>
       </c>
       <c r="N2" t="n">
         <v>0.2</v>
@@ -20479,16 +20479,16 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>169218.0588400939</v>
+        <v>169333.9172819833</v>
       </c>
       <c r="Q2" t="n">
-        <v>176255.095877131</v>
+        <v>176370.9543190204</v>
       </c>
       <c r="R2" t="n">
-        <v>4017.835141733316</v>
+        <v>4013.964820269089</v>
       </c>
       <c r="S2" t="n">
-        <v>4184.919286858772</v>
+        <v>4180.773806672917</v>
       </c>
       <c r="T2" t="n">
         <v>20</v>
@@ -20498,14 +20498,14 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W2" t="n">
-        <v>112.8358942581749</v>
+        <v>110.769405</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="3">
@@ -20525,10 +20525,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>31.53801554024096</v>
+        <v>31.7027399</v>
       </c>
       <c r="E3" t="n">
-        <v>496.99588164</v>
+        <v>499.2745676166667</v>
       </c>
       <c r="F3" t="n">
         <v>503.204</v>
@@ -20540,19 +20540,19 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.9876628199298892</v>
+        <v>0.9921911741891296</v>
       </c>
       <c r="J3" t="n">
-        <v>1.012491287331224</v>
+        <v>1.007870283483677</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3876628199298892</v>
+        <v>0.3921911741891295</v>
       </c>
       <c r="M3" t="n">
-        <v>0.7124912873312235</v>
+        <v>0.7078702834836768</v>
       </c>
       <c r="N3" t="n">
         <v>0.2</v>
@@ -20563,16 +20563,16 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>120549.0972492752</v>
+        <v>120823.8025732333</v>
       </c>
       <c r="Q3" t="n">
-        <v>127586.1342863122</v>
+        <v>127860.8396102704</v>
       </c>
       <c r="R3" t="n">
-        <v>3822.342502668262</v>
+        <v>3811.147016136399</v>
       </c>
       <c r="S3" t="n">
-        <v>4045.471222611282</v>
+        <v>4033.116380905311</v>
       </c>
       <c r="T3" t="n">
         <v>20</v>
@@ -20582,14 +20582,14 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W3" t="n">
-        <v>2.450200000000002</v>
+        <v>2.4502</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="4">
@@ -20609,10 +20609,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>19.80174807036145</v>
+        <v>19.93824174</v>
       </c>
       <c r="E4" t="n">
-        <v>334.6441816399999</v>
+        <v>336.53234307</v>
       </c>
       <c r="F4" t="n">
         <v>337.444</v>
@@ -20624,19 +20624,19 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9917028651865196</v>
+        <v>0.9972983460070414</v>
       </c>
       <c r="J4" t="n">
-        <v>1.008366553233584</v>
+        <v>1.00270897269987</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3917028651865197</v>
+        <v>0.3972983460070414</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7083665532335834</v>
+        <v>0.7027089726998701</v>
       </c>
       <c r="N4" t="n">
         <v>0.2</v>
@@ -20647,16 +20647,16 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>81085.71519867277</v>
+        <v>81313.34114174001</v>
       </c>
       <c r="Q4" t="n">
-        <v>88122.75223570981</v>
+        <v>88350.37817877704</v>
       </c>
       <c r="R4" t="n">
-        <v>4094.876619506082</v>
+        <v>4078.26037030184</v>
       </c>
       <c r="S4" t="n">
-        <v>4450.251155735528</v>
+        <v>4431.202075433209</v>
       </c>
       <c r="T4" t="n">
         <v>20</v>
@@ -20666,14 +20666,14 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="5">
@@ -20693,10 +20693,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15.08403817127711</v>
+        <v>15.24396773</v>
       </c>
       <c r="E5" t="n">
-        <v>269.382528036</v>
+        <v>271.5948859316667</v>
       </c>
       <c r="F5" t="n">
         <v>272.804</v>
@@ -20708,19 +20708,19 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0.98745813124441</v>
+        <v>0.9955678286669796</v>
       </c>
       <c r="J5" t="n">
-        <v>1.012701165101334</v>
+        <v>1.004451902929562</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0.38745813124441</v>
+        <v>0.3955678286669796</v>
       </c>
       <c r="M5" t="n">
-        <v>0.712701165101334</v>
+        <v>0.7044519029295622</v>
       </c>
       <c r="N5" t="n">
         <v>0.2</v>
@@ -20731,16 +20731,16 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>65461.34765696646</v>
+        <v>65728.05685106333</v>
       </c>
       <c r="Q5" t="n">
-        <v>72498.3846940035</v>
+        <v>72765.09388810037</v>
       </c>
       <c r="R5" t="n">
-        <v>4339.776054241057</v>
+        <v>4311.74206185907</v>
       </c>
       <c r="S5" t="n">
-        <v>4806.298145814447</v>
+        <v>4773.369714296841</v>
       </c>
       <c r="T5" t="n">
         <v>20</v>
@@ -20750,14 +20750,14 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W5" t="n">
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="6">
@@ -20777,10 +20777,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>37.78000099520155</v>
+        <v>37.9998124</v>
       </c>
       <c r="E6" t="n">
-        <v>583.343347100288</v>
+        <v>586.3840705333333</v>
       </c>
       <c r="F6" t="n">
         <v>658.904</v>
@@ -20792,19 +20792,19 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8853237301644671</v>
+        <v>0.889938550279454</v>
       </c>
       <c r="J6" t="n">
-        <v>1.129530324251254</v>
+        <v>1.123673089210469</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2853237301644671</v>
+        <v>0.289938550279454</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8295303242512537</v>
+        <v>0.8236730892104687</v>
       </c>
       <c r="N6" t="n">
         <v>0.2</v>
@@ -20815,16 +20815,16 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>146556.8483263311</v>
+        <v>146923.4204790667</v>
       </c>
       <c r="Q6" t="n">
-        <v>153593.8853633682</v>
+        <v>153960.4575161037</v>
       </c>
       <c r="R6" t="n">
-        <v>3879.217693640224</v>
+        <v>3866.424890009896</v>
       </c>
       <c r="S6" t="n">
-        <v>4065.481241857992</v>
+        <v>4051.610989429615</v>
       </c>
       <c r="T6" t="n">
         <v>20</v>
@@ -20834,14 +20834,14 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W6" t="n">
-        <v>67.20108868896887</v>
+        <v>66.0522835</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="7">
@@ -20861,10 +20861,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24.45102674983387</v>
+        <v>24.47100939</v>
       </c>
       <c r="E7" t="n">
-        <v>398.959203372702</v>
+        <v>399.235628895</v>
       </c>
       <c r="F7" t="n">
         <v>400.3440000000001</v>
@@ -20876,19 +20876,19 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9965409831862146</v>
+        <v>0.9972314531877584</v>
       </c>
       <c r="J7" t="n">
-        <v>1.003471023141192</v>
+        <v>1.002776232943106</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3965409831862146</v>
+        <v>0.3972314531877584</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7034710231411918</v>
+        <v>0.7027762329431062</v>
       </c>
       <c r="N7" t="n">
         <v>0.2</v>
@@ -20899,16 +20899,16 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>93301.36227647297</v>
+        <v>93334.68665939</v>
       </c>
       <c r="Q7" t="n">
-        <v>100338.39931351</v>
+        <v>100371.723696427</v>
       </c>
       <c r="R7" t="n">
-        <v>3815.846394961998</v>
+        <v>3814.092225289689</v>
       </c>
       <c r="S7" t="n">
-        <v>4103.647684823368</v>
+        <v>4101.658501158666</v>
       </c>
       <c r="T7" t="n">
         <v>20</v>
@@ -20918,14 +20918,14 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="8">
@@ -20945,10 +20945,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>12.41382401123147</v>
+        <v>12.48514207</v>
       </c>
       <c r="E8" t="n">
-        <v>232.444565488702</v>
+        <v>233.4311309683333</v>
       </c>
       <c r="F8" t="n">
         <v>234.584</v>
@@ -20960,19 +20960,19 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.9908798788012052</v>
+        <v>0.995085474577692</v>
       </c>
       <c r="J8" t="n">
-        <v>1.009204063372271</v>
+        <v>1.004938797267033</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3908798788012052</v>
+        <v>0.395085474577692</v>
       </c>
       <c r="M8" t="n">
-        <v>0.7092040633722712</v>
+        <v>0.7049387972670322</v>
       </c>
       <c r="N8" t="n">
         <v>0.2</v>
@@ -20983,16 +20983,16 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>53336.12050939701</v>
+        <v>53455.05525873667</v>
       </c>
       <c r="Q8" t="n">
-        <v>60373.15754643404</v>
+        <v>60492.09229577371</v>
       </c>
       <c r="R8" t="n">
-        <v>4296.510121388937</v>
+        <v>4281.493551217289</v>
       </c>
       <c r="S8" t="n">
-        <v>4863.381137980621</v>
+        <v>4845.1264676537</v>
       </c>
       <c r="T8" t="n">
         <v>20</v>
@@ -21002,14 +21002,14 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="9">
@@ -21029,10 +21029,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7.476212876356526</v>
+        <v>7.75586028</v>
       </c>
       <c r="E9" t="n">
-        <v>164.1409447895986</v>
+        <v>168.00939954</v>
       </c>
       <c r="F9" t="n">
         <v>169.944</v>
@@ -21044,19 +21044,19 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0.9658531327354812</v>
+        <v>0.9886162473520688</v>
       </c>
       <c r="J9" t="n">
-        <v>1.035354098989986</v>
+        <v>1.011514834677684</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3658531327354811</v>
+        <v>0.3886162473520689</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7353540989899865</v>
+        <v>0.7115148346776836</v>
       </c>
       <c r="N9" t="n">
         <v>0.2</v>
@@ -21067,16 +21067,16 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>37345.0310068039</v>
+        <v>37811.38966028</v>
       </c>
       <c r="Q9" t="n">
-        <v>44382.06804384093</v>
+        <v>44848.42669731704</v>
       </c>
       <c r="R9" t="n">
-        <v>4995.180263647562</v>
+        <v>4875.202530115718</v>
       </c>
       <c r="S9" t="n">
-        <v>5936.437174521732</v>
+        <v>5782.521226299997</v>
       </c>
       <c r="T9" t="n">
         <v>20</v>
@@ -21086,14 +21086,14 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="10">
@@ -21113,10 +21113,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>44.21697480464732</v>
+        <v>44.21697486</v>
       </c>
       <c r="E10" t="n">
-        <v>672.3881514642879</v>
+        <v>672.3881512299999</v>
       </c>
       <c r="F10" t="n">
         <v>780.8399999999999</v>
@@ -21128,19 +21128,19 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8611087437430049</v>
+        <v>0.8611087434429588</v>
       </c>
       <c r="J10" t="n">
-        <v>1.161293515210718</v>
+        <v>1.161293515615361</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2611087437430049</v>
+        <v>0.2611087434429588</v>
       </c>
       <c r="M10" t="n">
-        <v>0.8612935152107184</v>
+        <v>0.8612935156153614</v>
       </c>
       <c r="N10" t="n">
         <v>0.2</v>
@@ -21151,16 +21151,16 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>175581.9749825502</v>
+        <v>175581.97507486</v>
       </c>
       <c r="Q10" t="n">
-        <v>182619.0120195872</v>
+        <v>182619.0121118971</v>
       </c>
       <c r="R10" t="n">
-        <v>3970.917860352944</v>
+        <v>3970.917857469638</v>
       </c>
       <c r="S10" t="n">
-        <v>4130.065723094052</v>
+        <v>4130.065720011517</v>
       </c>
       <c r="T10" t="n">
         <v>20</v>
@@ -21170,14 +21170,14 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W10" t="n">
-        <v>103.8897580185268</v>
+        <v>102.651095</v>
       </c>
       <c r="X10" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="11">
@@ -21197,10 +21197,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>33.31408379063093</v>
+        <v>33.31408380000001</v>
       </c>
       <c r="E11" t="n">
-        <v>521.5648257703945</v>
+        <v>521.5648249000001</v>
       </c>
       <c r="F11" t="n">
         <v>522.28</v>
@@ -21212,19 +21212,19 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0.9986306689331288</v>
+        <v>0.9986306672666004</v>
       </c>
       <c r="J11" t="n">
-        <v>1.001371208705551</v>
+        <v>1.001371210376653</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3986306689331288</v>
+        <v>0.3986306672666004</v>
       </c>
       <c r="M11" t="n">
-        <v>0.7013712087055508</v>
+        <v>0.7013712103766525</v>
       </c>
       <c r="N11" t="n">
         <v>0.2</v>
@@ -21235,16 +21235,16 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>126372.3870681755</v>
+        <v>126372.3870838</v>
       </c>
       <c r="Q11" t="n">
-        <v>133409.4241052126</v>
+        <v>133409.424120837</v>
       </c>
       <c r="R11" t="n">
-        <v>3793.362226690317</v>
+        <v>3793.362226092497</v>
       </c>
       <c r="S11" t="n">
-        <v>4004.595322016086</v>
+        <v>4004.595321358861</v>
       </c>
       <c r="T11" t="n">
         <v>20</v>
@@ -21254,14 +21254,14 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="12">
@@ -21281,10 +21281,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>21.38313253012048</v>
+        <v>21.38313252</v>
       </c>
       <c r="E12" t="n">
-        <v>356.52</v>
+        <v>356.51999886</v>
       </c>
       <c r="F12" t="n">
         <v>356.52</v>
@@ -21296,19 +21296,19 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>0.9999999968024232</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>1.000000003197577</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0.3999999999999999</v>
+        <v>0.3999999968024232</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7000000000000002</v>
+        <v>0.7000000031975766</v>
       </c>
       <c r="N12" t="n">
         <v>0.2</v>
@@ -21319,16 +21319,16 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>86584.3373493976</v>
+        <v>86584.33733252001</v>
       </c>
       <c r="Q12" t="n">
-        <v>93621.37438643465</v>
+        <v>93621.37436955704</v>
       </c>
       <c r="R12" t="n">
-        <v>4049.188640973631</v>
+        <v>4049.188642100789</v>
       </c>
       <c r="S12" t="n">
-        <v>4378.281538243224</v>
+        <v>4378.281539526139</v>
       </c>
       <c r="T12" t="n">
         <v>20</v>
@@ -21338,14 +21338,14 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="13">
@@ -21365,10 +21365,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>16.71036144578313</v>
+        <v>16.71036152</v>
       </c>
       <c r="E13" t="n">
-        <v>291.88</v>
+        <v>291.8800000266667</v>
       </c>
       <c r="F13" t="n">
         <v>291.88</v>
@@ -21380,19 +21380,19 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>1.000000000091362</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0.9999999999086382</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4</v>
+        <v>0.4000000000913618</v>
       </c>
       <c r="M13" t="n">
-        <v>0.7</v>
+        <v>0.6999999999086381</v>
       </c>
       <c r="N13" t="n">
         <v>0.2</v>
@@ -21403,16 +21403,16 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>71034.91277108435</v>
+        <v>71034.91289485335</v>
       </c>
       <c r="Q13" t="n">
-        <v>78071.94980812138</v>
+        <v>78071.94993189038</v>
       </c>
       <c r="R13" t="n">
-        <v>4250.950106708197</v>
+        <v>4250.950095234884</v>
       </c>
       <c r="S13" t="n">
-        <v>4672.06828897306</v>
+        <v>4672.068275629406</v>
       </c>
       <c r="T13" t="n">
         <v>20</v>
@@ -21422,14 +21422,14 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="14">
@@ -21449,10 +21449,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>47.6905664648928</v>
+        <v>47.7401555</v>
       </c>
       <c r="E14" t="n">
-        <v>720.4395027643504</v>
+        <v>721.1254834166666</v>
       </c>
       <c r="F14" t="n">
         <v>876.924</v>
@@ -21464,19 +21464,19 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8215529541492198</v>
+        <v>0.8223352119643967</v>
       </c>
       <c r="J14" t="n">
-        <v>1.217206991892051</v>
+        <v>1.216049106800616</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0.2215529541492198</v>
+        <v>0.2223352119643967</v>
       </c>
       <c r="M14" t="n">
-        <v>0.9172069918920508</v>
+        <v>0.916049106800616</v>
       </c>
       <c r="N14" t="n">
         <v>0.2</v>
@@ -21487,16 +21487,16 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>195787.3680079529</v>
+        <v>195870.0659888333</v>
       </c>
       <c r="Q14" t="n">
-        <v>202824.4050449899</v>
+        <v>202907.1030258704</v>
       </c>
       <c r="R14" t="n">
-        <v>4105.36889202356</v>
+        <v>4102.836782524374</v>
       </c>
       <c r="S14" t="n">
-        <v>4252.925055824158</v>
+        <v>4250.239675609569</v>
       </c>
       <c r="T14" t="n">
         <v>20</v>
@@ -21506,14 +21506,14 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W14" t="n">
-        <v>151.1617553556355</v>
+        <v>148.819294</v>
       </c>
       <c r="X14" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="15">
@@ -21533,10 +21533,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>40.12480379748507</v>
+        <v>40.17414683</v>
       </c>
       <c r="E15" t="n">
-        <v>615.7797858652102</v>
+        <v>616.4623634816667</v>
       </c>
       <c r="F15" t="n">
         <v>618.364</v>
@@ -21548,19 +21548,19 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0.9958208852151972</v>
+        <v>0.9969247295794492</v>
       </c>
       <c r="J15" t="n">
-        <v>1.004196653079735</v>
+        <v>1.003084756882145</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0.3958208852151972</v>
+        <v>0.3969247295794493</v>
       </c>
       <c r="M15" t="n">
-        <v>0.704196653079735</v>
+        <v>0.7030847568821448</v>
       </c>
       <c r="N15" t="n">
         <v>0.2</v>
@@ -21571,16 +21571,16 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>152142.9977996059</v>
+        <v>152225.2855301633</v>
       </c>
       <c r="Q15" t="n">
-        <v>159180.034836643</v>
+        <v>159262.3225672004</v>
       </c>
       <c r="R15" t="n">
-        <v>3791.744342663724</v>
+        <v>3789.135489903902</v>
       </c>
       <c r="S15" t="n">
-        <v>3967.123070309443</v>
+        <v>3964.298812396221</v>
       </c>
       <c r="T15" t="n">
         <v>20</v>
@@ -21590,14 +21590,14 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W15" t="n">
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="16">
@@ -21617,10 +21617,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>28.27929318101204</v>
+        <v>28.31929618</v>
       </c>
       <c r="E16" t="n">
-        <v>451.916889004</v>
+        <v>452.4702628233333</v>
       </c>
       <c r="F16" t="n">
         <v>452.604</v>
@@ -21632,19 +21632,19 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0.9984818715786868</v>
+        <v>0.9997045161406732</v>
       </c>
       <c r="J16" t="n">
-        <v>1.001520436639388</v>
+        <v>1.000295571195844</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0.3984818715786867</v>
+        <v>0.3997045161406732</v>
       </c>
       <c r="M16" t="n">
-        <v>0.7015204366393883</v>
+        <v>0.7002955711958443</v>
       </c>
       <c r="N16" t="n">
         <v>0.2</v>
@@ -21655,16 +21655,16 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>112497.4345948678</v>
+        <v>112564.1462628467</v>
       </c>
       <c r="Q16" t="n">
-        <v>119534.4716319048</v>
+        <v>119601.1832998837</v>
       </c>
       <c r="R16" t="n">
-        <v>3978.085091264002</v>
+        <v>3974.821462630244</v>
       </c>
       <c r="S16" t="n">
-        <v>4226.925717937161</v>
+        <v>4223.310584404634</v>
       </c>
       <c r="T16" t="n">
         <v>20</v>
@@ -21674,14 +21674,14 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W16" t="n">
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="17">
@@ -21701,10 +21701,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>23.60652209667469</v>
+        <v>23.64652497</v>
       </c>
       <c r="E17" t="n">
-        <v>387.276889004</v>
+        <v>387.830261085</v>
       </c>
       <c r="F17" t="n">
         <v>387.964</v>
@@ -21716,19 +21716,19 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.9982289310451484</v>
+        <v>0.9996552800904208</v>
       </c>
       <c r="J17" t="n">
-        <v>1.001774211205237</v>
+        <v>1.000344838782373</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0.3982289310451483</v>
+        <v>0.3996552800904208</v>
       </c>
       <c r="M17" t="n">
-        <v>0.7017742112052365</v>
+        <v>0.700344838782373</v>
       </c>
       <c r="N17" t="n">
         <v>0.2</v>
@@ -21739,16 +21739,16 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>96948.0100165545</v>
+        <v>97014.72147497001</v>
       </c>
       <c r="Q17" t="n">
-        <v>103985.0470535915</v>
+        <v>104051.758512007</v>
       </c>
       <c r="R17" t="n">
-        <v>4106.831562037297</v>
+        <v>4102.705221932235</v>
       </c>
       <c r="S17" t="n">
-        <v>4404.928715367151</v>
+        <v>4400.298083714878</v>
       </c>
       <c r="T17" t="n">
         <v>20</v>
@@ -21758,14 +21758,14 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W17" t="n">
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="18">
@@ -21785,10 +21785,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>44.67268564802082</v>
+        <v>44.67268558</v>
       </c>
       <c r="E18" t="n">
-        <v>678.6921514642879</v>
+        <v>678.6921495233333</v>
       </c>
       <c r="F18" t="n">
         <v>819.4200000000001</v>
@@ -21800,19 +21800,19 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8282591973155254</v>
+        <v>0.8282591949468322</v>
       </c>
       <c r="J18" t="n">
-        <v>1.207351518994422</v>
+        <v>1.20735152244726</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0.2282591973155254</v>
+        <v>0.2282591949468322</v>
       </c>
       <c r="M18" t="n">
-        <v>0.9073515189944216</v>
+        <v>0.90735152244726</v>
       </c>
       <c r="N18" t="n">
         <v>0.2</v>
@@ -21823,16 +21823,16 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>182128.9487656828</v>
+        <v>182128.9486522467</v>
       </c>
       <c r="Q18" t="n">
-        <v>189165.9858027197</v>
+        <v>189165.9856892837</v>
       </c>
       <c r="R18" t="n">
-        <v>4076.964393873458</v>
+        <v>4076.964397541973</v>
       </c>
       <c r="S18" t="n">
-        <v>4234.488772248252</v>
+        <v>4234.488776156621</v>
       </c>
       <c r="T18" t="n">
         <v>20</v>
@@ -21842,14 +21842,14 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W18" t="n">
-        <v>136.14439980008</v>
+        <v>134.05329</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="19">
@@ -21869,10 +21869,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>35.97400601109744</v>
+        <v>35.97400591</v>
       </c>
       <c r="E19" t="n">
-        <v>558.360416486848</v>
+        <v>558.3604140883333</v>
       </c>
       <c r="F19" t="n">
         <v>560.8599999999999</v>
@@ -21884,19 +21884,19 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0.9955433022266664</v>
+        <v>0.9955432979501718</v>
       </c>
       <c r="J19" t="n">
-        <v>1.00447664884427</v>
+        <v>1.004476653159139</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3955433022266663</v>
+        <v>0.3955432979501718</v>
       </c>
       <c r="M19" t="n">
-        <v>0.70447664884427</v>
+        <v>0.7044766531591389</v>
       </c>
       <c r="N19" t="n">
         <v>0.2</v>
@@ -21907,16 +21907,16 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>136595.2506911735</v>
+        <v>136595.2505225767</v>
       </c>
       <c r="Q19" t="n">
-        <v>143632.2877282105</v>
+        <v>143632.2875596137</v>
       </c>
       <c r="R19" t="n">
-        <v>3797.054202110155</v>
+        <v>3797.054208094354</v>
       </c>
       <c r="S19" t="n">
-        <v>3992.668697611885</v>
+        <v>3992.668704145819</v>
       </c>
       <c r="T19" t="n">
         <v>20</v>
@@ -21926,14 +21926,14 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W19" t="n">
-        <v>0.7421999999999969</v>
+        <v>0.7422</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="20">
@@ -21953,10 +21953,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>24.17204819277108</v>
+        <v>24.17204819</v>
       </c>
       <c r="E20" t="n">
-        <v>395.1</v>
+        <v>395.0999989616667</v>
       </c>
       <c r="F20" t="n">
         <v>395.1</v>
@@ -21968,19 +21968,19 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0.9999999973719732</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>1.000000002628027</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0.4</v>
+        <v>0.3999999973719733</v>
       </c>
       <c r="M20" t="n">
-        <v>0.7</v>
+        <v>0.7000000026280266</v>
       </c>
       <c r="N20" t="n">
         <v>0.2</v>
@@ -21991,16 +21991,16 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>97022.31903614456</v>
+        <v>97022.31903152334</v>
       </c>
       <c r="Q20" t="n">
-        <v>104059.3560731816</v>
+        <v>104059.3560685604</v>
       </c>
       <c r="R20" t="n">
-        <v>4013.822836294037</v>
+        <v>4013.822836563</v>
       </c>
       <c r="S20" t="n">
-        <v>4304.945747390232</v>
+        <v>4304.945747692569</v>
       </c>
       <c r="T20" t="n">
         <v>20</v>
@@ -22010,14 +22010,14 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W20" t="n">
         <v>0</v>
       </c>
       <c r="X20" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="21">
@@ -22037,10 +22037,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>19.49927710843373</v>
+        <v>19.49927706</v>
       </c>
       <c r="E21" t="n">
-        <v>330.4599999999999</v>
+        <v>330.45999833</v>
       </c>
       <c r="F21" t="n">
         <v>330.4599999999999</v>
@@ -22052,19 +22052,19 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0.9999999949464384</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>1.000000005053561</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.3999999949464385</v>
       </c>
       <c r="M21" t="n">
-        <v>0.7</v>
+        <v>0.7000000050535613</v>
       </c>
       <c r="N21" t="n">
         <v>0.2</v>
@@ -22075,16 +22075,16 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>81472.89445783132</v>
+        <v>81472.89437706</v>
       </c>
       <c r="Q21" t="n">
-        <v>88509.93149486836</v>
+        <v>88509.93141409704</v>
       </c>
       <c r="R21" t="n">
-        <v>4178.252045179309</v>
+        <v>4178.252051415285</v>
       </c>
       <c r="S21" t="n">
-        <v>4539.139117961787</v>
+        <v>4539.139125094161</v>
       </c>
       <c r="T21" t="n">
         <v>20</v>
@@ -22094,14 +22094,14 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W21" t="n">
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="22">
@@ -22121,10 +22121,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>42.08169769621359</v>
+        <v>42.08169784</v>
       </c>
       <c r="E22" t="n">
-        <v>642.850151464288</v>
+        <v>642.8501524533334</v>
       </c>
       <c r="F22" t="n">
         <v>715.76</v>
@@ -22136,19 +22136,19 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0.898136458399866</v>
+        <v>0.8981364597816774</v>
       </c>
       <c r="J22" t="n">
-        <v>1.113416553406167</v>
+        <v>1.11341655169314</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>0.298136458399866</v>
+        <v>0.2981364597816774</v>
       </c>
       <c r="M22" t="n">
-        <v>0.8134165534061668</v>
+        <v>0.8134165516931402</v>
       </c>
       <c r="N22" t="n">
         <v>0.2</v>
@@ -22159,16 +22159,16 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>162259.0445247189</v>
+        <v>162259.0447645067</v>
       </c>
       <c r="Q22" t="n">
-        <v>169296.0815617559</v>
+        <v>169296.0818015437</v>
       </c>
       <c r="R22" t="n">
-        <v>3855.810326286302</v>
+        <v>3855.810318809768</v>
       </c>
       <c r="S22" t="n">
-        <v>4023.033547360632</v>
+        <v>4023.033539312722</v>
       </c>
       <c r="T22" t="n">
         <v>20</v>
@@ -22178,14 +22178,14 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W22" t="n">
-        <v>68.40251787449543</v>
+        <v>67.2486401</v>
       </c>
       <c r="X22" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="23">
@@ -22205,10 +22205,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28.66120481927711</v>
+        <v>28.66120499</v>
       </c>
       <c r="E23" t="n">
-        <v>457.2000000000001</v>
+        <v>457.2000013616667</v>
       </c>
       <c r="F23" t="n">
         <v>457.2000000000001</v>
@@ -22220,19 +22220,19 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>1.000000002978273</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>0.9999999970217264</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>0.4</v>
+        <v>0.4000000029782734</v>
       </c>
       <c r="M23" t="n">
-        <v>0.7</v>
+        <v>0.6999999970217265</v>
       </c>
       <c r="N23" t="n">
         <v>0.2</v>
@@ -22243,16 +22243,16 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>108850.9359036144</v>
+        <v>108850.9361883233</v>
       </c>
       <c r="Q23" t="n">
-        <v>115887.9729406515</v>
+        <v>115887.9732253604</v>
       </c>
       <c r="R23" t="n">
-        <v>3797.849273607747</v>
+        <v>3797.849260919135</v>
       </c>
       <c r="S23" t="n">
-        <v>4043.374089518627</v>
+        <v>4043.374075367526</v>
       </c>
       <c r="T23" t="n">
         <v>20</v>
@@ -22262,14 +22262,14 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W23" t="n">
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="24">
@@ -22289,10 +22289,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>16.67855421686747</v>
+        <v>16.67855424</v>
       </c>
       <c r="E24" t="n">
-        <v>291.44</v>
+        <v>291.43999932</v>
       </c>
       <c r="F24" t="n">
         <v>291.44</v>
@@ -22304,19 +22304,19 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0.999999997666758</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>1.000000002333242</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4</v>
+        <v>0.3999999976667581</v>
       </c>
       <c r="M24" t="n">
-        <v>0.7</v>
+        <v>0.700000002333242</v>
       </c>
       <c r="N24" t="n">
         <v>0.2</v>
@@ -22327,16 +22327,16 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>68976.66891566265</v>
+        <v>68976.66895424</v>
       </c>
       <c r="Q24" t="n">
-        <v>76013.70595269969</v>
+        <v>76013.70599127703</v>
       </c>
       <c r="R24" t="n">
-        <v>4135.650369856681</v>
+        <v>4135.65036643368</v>
       </c>
       <c r="S24" t="n">
-        <v>4557.571655451105</v>
+        <v>4557.571651442915</v>
       </c>
       <c r="T24" t="n">
         <v>20</v>
@@ -22346,14 +22346,14 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W24" t="n">
         <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
     <row r="25">
@@ -22373,10 +22373,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11.90163254974843</v>
+        <v>11.93913026</v>
       </c>
       <c r="E25" t="n">
-        <v>225.35925027152</v>
+        <v>225.8779675966667</v>
       </c>
       <c r="F25" t="n">
         <v>226.8</v>
@@ -22388,19 +22388,19 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0.993647487969665</v>
+        <v>0.9959346013962376</v>
       </c>
       <c r="J25" t="n">
-        <v>1.006393124430189</v>
+        <v>1.004081993534579</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>0.393647487969665</v>
+        <v>0.3959346013962375</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7063931244301893</v>
+        <v>0.7040819935345786</v>
       </c>
       <c r="N25" t="n">
         <v>0.2</v>
@@ -22411,16 +22411,16 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>53253.55588213047</v>
+        <v>53316.08956359333</v>
       </c>
       <c r="Q25" t="n">
-        <v>60290.59291916751</v>
+        <v>60353.12660063037</v>
       </c>
       <c r="R25" t="n">
-        <v>4474.474880612584</v>
+        <v>4465.659424306619</v>
       </c>
       <c r="S25" t="n">
-        <v>5065.741415486893</v>
+        <v>5055.06894441324</v>
       </c>
       <c r="T25" t="n">
         <v>20</v>
@@ -22430,14 +22430,14 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>discrete_storage_fallback</t>
+          <t>pulp_milp_optimal</t>
         </is>
       </c>
       <c r="W25" t="n">
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>0</v>
+        <v>1e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>